<commit_message>
fix(seeding): update data seeding for lamaran, surat keluar, and surat masuk with proper mapping and sorting
</commit_message>
<xml_diff>
--- a/data_raw/lamaran.xlsx
+++ b/data_raw/lamaran.xlsx
@@ -5,18 +5,29 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookair/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookair/self-projects/in-hc/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FFFF988-36DF-7F45-B432-5018733C3705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8519B64-C4A7-3549-9A55-A7FC956DE80A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LAMARAN" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="pxFc6cUxk9mDnqipqP8g4uk0hlMFybPm6cHmKZ8evbI="/>
     </ext>
@@ -492,12 +503,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -559,22 +572,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -679,25 +676,41 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="3">
     <tableStyle name="LAMARAN-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="8"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
-      <tableStyleElement type="secondRowStripe" dxfId="9"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
+      <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
     <tableStyle name="SURAT MASUK-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="SURAT KELUAR-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>

</xml_diff>